<commit_message>
titles and topics format
</commit_message>
<xml_diff>
--- a/SCOTUS Focus Group Responses copy.xlsx
+++ b/SCOTUS Focus Group Responses copy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://brennancenterny-my.sharepoint.com/personal/sanchezg_brennan_law_nyu_edu/Documents/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="783" documentId="8_{257FA1E6-886D-2E4B-AFC6-BC55E68113DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{697BE419-2D59-F947-9053-1FECB06FFBA6}"/>
+  <xr:revisionPtr revIDLastSave="812" documentId="8_{257FA1E6-886D-2E4B-AFC6-BC55E68113DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95FD8D7B-B0A6-DD43-94D3-90130C53E20F}"/>
   <bookViews>
-    <workbookView xWindow="220" yWindow="760" windowWidth="28980" windowHeight="15320" activeTab="3" xr2:uid="{E594D9D5-8148-944B-9F41-235101522376}"/>
+    <workbookView xWindow="220" yWindow="760" windowWidth="28980" windowHeight="15320" xr2:uid="{E594D9D5-8148-944B-9F41-235101522376}"/>
   </bookViews>
   <sheets>
     <sheet name="Participants" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="310">
   <si>
     <t>Holly</t>
   </si>
@@ -1042,32 +1042,6 @@
   </si>
   <si>
     <t>Vincent (D, NY)</t>
-  </si>
-  <si>
-    <r>
-      <t>Jeremy (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>N/A</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, TX)</t>
-    </r>
   </si>
   <si>
     <t>They are appointed by the president at the time, and they serve in the term for the rest of their life until they don't want to anymore. And literally any decision that they make is final for the country.</t>
@@ -2316,7 +2290,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -2463,11 +2437,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2517,22 +2502,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2557,6 +2526,33 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2578,6 +2574,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2897,7 +2897,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A4C20F6-087B-DE40-82F4-FDC01EE5D7C0}">
-  <dimension ref="B1:E9"/>
+  <dimension ref="C1:E9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="30" customWidth="1"/>
@@ -2906,96 +2906,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="C1" s="33" t="s">
+      <c r="C1" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="D1" s="33" t="s">
+      <c r="D1" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="E1" s="33" t="s">
+      <c r="E1" s="27" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="2" spans="3:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="C2" s="34" t="s">
+      <c r="C2" s="28" t="s">
+        <v>289</v>
+      </c>
+      <c r="D2" s="28" t="s">
         <v>290</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="E2" s="29" t="s">
         <v>291</v>
       </c>
-      <c r="E2" s="35" t="s">
+    </row>
+    <row r="3" spans="3:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="C3" s="28" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="3" spans="3:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="C3" s="34" t="s">
+      <c r="D3" s="30" t="s">
         <v>293</v>
       </c>
-      <c r="D3" s="36" t="s">
+      <c r="E3" s="29" t="s">
         <v>294</v>
       </c>
-      <c r="E3" s="35" t="s">
+    </row>
+    <row r="4" spans="3:5" ht="68" x14ac:dyDescent="0.2">
+      <c r="C4" s="28" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="4" spans="3:5" ht="68" x14ac:dyDescent="0.2">
-      <c r="C4" s="34" t="s">
+      <c r="D4" s="31" t="s">
         <v>296</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="E4" s="29" t="s">
         <v>297</v>
       </c>
-      <c r="E4" s="35" t="s">
+    </row>
+    <row r="5" spans="3:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="C5" s="28" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="5" spans="3:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="C5" s="34" t="s">
+      <c r="D5" s="28" t="s">
         <v>299</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="E5" s="29" t="s">
         <v>300</v>
       </c>
-      <c r="E5" s="35" t="s">
+    </row>
+    <row r="6" spans="3:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="C6" s="28" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="6" spans="3:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="C6" s="34" t="s">
+      <c r="D6" s="28" t="s">
         <v>302</v>
       </c>
-      <c r="D6" s="34" t="s">
+      <c r="E6" s="29" t="s">
         <v>303</v>
       </c>
-      <c r="E6" s="35" t="s">
+    </row>
+    <row r="7" spans="3:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="C7" s="28" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="7" spans="3:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="C7" s="34" t="s">
+      <c r="D7" s="30" t="s">
         <v>305</v>
       </c>
-      <c r="D7" s="36" t="s">
+      <c r="E7" s="29" t="s">
         <v>306</v>
       </c>
-      <c r="E7" s="35" t="s">
+    </row>
+    <row r="8" spans="3:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="C8" s="30" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="8" spans="3:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="C8" s="36" t="s">
+      <c r="D8" s="32"/>
+      <c r="E8" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="D8" s="38"/>
-      <c r="E8" s="35" t="s">
+    </row>
+    <row r="9" spans="3:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="34" t="s">
         <v>309</v>
-      </c>
-    </row>
-    <row r="9" spans="3:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="40" t="s">
-        <v>310</v>
       </c>
     </row>
   </sheetData>
@@ -3094,7 +3094,7 @@
     <row r="12" spans="7:18" x14ac:dyDescent="0.2">
       <c r="P12" s="20"/>
       <c r="Q12" s="21" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13" spans="7:18" x14ac:dyDescent="0.2">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="P14" s="20"/>
       <c r="Q14" s="21" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="15" spans="7:18" x14ac:dyDescent="0.2">
@@ -3167,7 +3167,7 @@
     </row>
     <row r="21" spans="4:17" x14ac:dyDescent="0.2">
       <c r="G21" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="22" spans="4:17" x14ac:dyDescent="0.2">
@@ -3177,7 +3177,7 @@
     </row>
     <row r="23" spans="4:17" x14ac:dyDescent="0.2">
       <c r="G23" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="24" spans="4:17" x14ac:dyDescent="0.2">
@@ -3245,173 +3245,190 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3C5F046-F19C-3A40-A16A-7CDF84CFAD9D}">
-  <dimension ref="D2:I10"/>
+  <dimension ref="D2:I11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" customWidth="1"/>
+    <col min="7" max="7" width="9.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.6640625" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="4:9" x14ac:dyDescent="0.2">
-      <c r="D2" s="30" t="s">
+      <c r="D2" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="E2" s="31"/>
-      <c r="F2" s="30" t="s">
+      <c r="E2" s="36"/>
+      <c r="F2" s="35" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="30"/>
-      <c r="H2" s="32" t="s">
+      <c r="G2" s="35"/>
+      <c r="H2" s="37" t="s">
         <v>62</v>
       </c>
-      <c r="I2" s="30"/>
+      <c r="I2" s="35"/>
     </row>
     <row r="3" spans="4:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="D3" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="E3" s="27" t="s">
+      <c r="D3" s="38" t="s">
+        <v>238</v>
+      </c>
+      <c r="E3" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="38" t="s">
+        <v>241</v>
+      </c>
+      <c r="G3" s="42" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="39" t="s">
+        <v>237</v>
+      </c>
+      <c r="I3" s="43" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="4:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="D4" s="40" t="s">
+        <v>245</v>
+      </c>
+      <c r="E4" s="42" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="38" t="s">
+        <v>251</v>
+      </c>
+      <c r="G4" s="42" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" s="39" t="s">
+        <v>235</v>
+      </c>
+      <c r="I4" s="43" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="4:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="D5" s="38" t="s">
+        <v>246</v>
+      </c>
+      <c r="E5" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="F5" s="38" t="s">
+        <v>244</v>
+      </c>
+      <c r="G5" s="42" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" s="39" t="s">
+        <v>239</v>
+      </c>
+      <c r="I5" s="43" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="4:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="D6" s="38" t="s">
+        <v>247</v>
+      </c>
+      <c r="E6" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="38" t="s">
+        <v>260</v>
+      </c>
+      <c r="G6" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="H6" s="39" t="s">
+        <v>240</v>
+      </c>
+      <c r="I6" s="43" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="4:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="D7" s="38" t="s">
+        <v>248</v>
+      </c>
+      <c r="E7" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7" s="38" t="s">
+        <v>272</v>
+      </c>
+      <c r="G7" s="42" t="s">
+        <v>37</v>
+      </c>
+      <c r="H7" s="39" t="s">
+        <v>242</v>
+      </c>
+      <c r="I7" s="43" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="4:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="D8" s="38" t="s">
+        <v>252</v>
+      </c>
+      <c r="E8" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" s="38" t="s">
+        <v>250</v>
+      </c>
+      <c r="G8" s="42" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" s="39" t="s">
+        <v>243</v>
+      </c>
+      <c r="I8" s="43" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="4:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D9" s="40" t="s">
         <v>253</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="E9" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="H3" s="29" t="s">
-        <v>239</v>
-      </c>
-      <c r="I3" s="28" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="4:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="D4" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="E4" s="27" t="s">
-        <v>33</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="G4" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="H4" s="29" t="s">
-        <v>242</v>
-      </c>
-      <c r="I4" s="28" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="4:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="D5" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="E5" s="27" t="s">
-        <v>34</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="G5" s="28" t="s">
-        <v>41</v>
-      </c>
-      <c r="H5" s="29" t="s">
-        <v>237</v>
-      </c>
-      <c r="I5" s="28" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="4:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="D6" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="E6" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="G6" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="H6" s="29" t="s">
+      <c r="F9" s="38"/>
+      <c r="G9" s="38"/>
+      <c r="H9" s="39" t="s">
+        <v>249</v>
+      </c>
+      <c r="I9" s="43" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="4:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="38"/>
+      <c r="H10" s="39" t="s">
         <v>236</v>
       </c>
-      <c r="I6" s="28" t="s">
+      <c r="I10" s="43" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="4:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="D7" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="E7" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="G7" s="28" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" s="29" t="s">
-        <v>243</v>
-      </c>
-      <c r="I7" s="28" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="4:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="D8" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="E8" s="27" t="s">
-        <v>37</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="G8" s="28" t="s">
-        <v>44</v>
-      </c>
-      <c r="H8" s="29" t="s">
-        <v>240</v>
-      </c>
-      <c r="I8" s="28" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="4:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="F9" s="29" t="s">
-        <v>245</v>
-      </c>
-      <c r="G9" s="28" t="s">
-        <v>39</v>
-      </c>
-      <c r="H9" s="29" t="s">
-        <v>235</v>
-      </c>
-      <c r="I9" s="28" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="4:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="H10" s="29" t="s">
-        <v>249</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>63</v>
-      </c>
+    <row r="11" spans="4:9" x14ac:dyDescent="0.2">
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="H3:I10">
+    <sortCondition ref="H3:H10"/>
+  </sortState>
   <mergeCells count="3">
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F2:G2"/>
@@ -3532,7 +3549,7 @@
         <v>86</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I2" s="9" t="s">
         <v>98</v>
@@ -3550,7 +3567,7 @@
       </c>
       <c r="O2" s="9"/>
       <c r="P2" s="9" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="Q2" s="8" t="s">
         <v>215</v>
@@ -3636,7 +3653,7 @@
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
       <c r="L4" s="9" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="M4" s="9"/>
       <c r="N4" s="9" t="s">
@@ -3646,7 +3663,7 @@
         <v>209</v>
       </c>
       <c r="P4" s="9" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="Q4" s="9"/>
       <c r="R4" s="9"/>
@@ -3674,7 +3691,7 @@
       <c r="F5" s="9"/>
       <c r="G5" s="9"/>
       <c r="H5" s="9" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I5" s="8" t="s">
         <v>222</v>
@@ -3736,7 +3753,7 @@
       </c>
       <c r="M6" s="9"/>
       <c r="N6" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="O6" s="8" t="s">
         <v>202</v>
@@ -3786,7 +3803,7 @@
       <c r="L7" s="9"/>
       <c r="M7" s="9"/>
       <c r="N7" s="9" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="O7" s="9"/>
       <c r="P7" s="9" t="s">
@@ -3796,7 +3813,7 @@
         <v>212</v>
       </c>
       <c r="R7" s="9" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="S7" s="9"/>
       <c r="T7" s="9"/>
@@ -3824,7 +3841,7 @@
       <c r="J8" s="9"/>
       <c r="K8" s="9"/>
       <c r="L8" s="8" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="M8" s="9"/>
       <c r="N8" s="9"/>
@@ -3858,7 +3875,7 @@
       <c r="J9" s="9"/>
       <c r="K9" s="9"/>
       <c r="L9" s="8" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="M9" s="9"/>
       <c r="N9" s="8" t="s">
@@ -3868,7 +3885,7 @@
         <v>208</v>
       </c>
       <c r="P9" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="Q9" s="8" t="s">
         <v>214</v>
@@ -3919,7 +3936,7 @@
         <v>161</v>
       </c>
       <c r="O10" s="18" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="P10" s="18" t="s">
         <v>231</v>
@@ -3974,7 +3991,7 @@
         <v>166</v>
       </c>
       <c r="P11" s="18" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="Q11" s="18" t="s">
         <v>169</v>
@@ -4027,7 +4044,7 @@
         <v>127</v>
       </c>
       <c r="Q12" s="18" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="R12" s="18"/>
       <c r="S12" s="18"/>
@@ -4084,7 +4101,7 @@
       <c r="R13" s="18"/>
       <c r="S13" s="18"/>
       <c r="T13" s="18" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="14" spans="1:20" s="10" customFormat="1" ht="238" x14ac:dyDescent="0.2">
@@ -4111,7 +4128,7 @@
         <v>143</v>
       </c>
       <c r="I14" s="18" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="J14" s="12" t="s">
         <v>149</v>
@@ -4152,7 +4169,7 @@
       </c>
       <c r="D15" s="18"/>
       <c r="E15" s="18" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F15" s="18"/>
       <c r="G15" s="18"/>
@@ -4173,7 +4190,7 @@
       <c r="N15" s="18"/>
       <c r="O15" s="18"/>
       <c r="P15" s="18" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="Q15" s="12" t="s">
         <v>171</v>
@@ -4217,11 +4234,11 @@
         <v>157</v>
       </c>
       <c r="N16" s="16" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="O16" s="16"/>
       <c r="P16" s="16" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Q16" s="15" t="s">
         <v>125</v>
@@ -4308,7 +4325,7 @@
         <v>96</v>
       </c>
       <c r="I18" s="16" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="J18" s="15" t="s">
         <v>102</v>
@@ -4324,13 +4341,13 @@
         <v>114</v>
       </c>
       <c r="O18" s="16" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="P18" s="16" t="s">
         <v>118</v>
       </c>
       <c r="Q18" s="16" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="R18" s="16" t="s">
         <v>128</v>
@@ -4339,7 +4356,7 @@
         <v>91</v>
       </c>
       <c r="T18" s="16" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19" spans="1:20" s="13" customFormat="1" ht="119" x14ac:dyDescent="0.2">
@@ -4360,7 +4377,7 @@
       </c>
       <c r="H19" s="16"/>
       <c r="I19" s="16" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J19" s="15" t="s">
         <v>100</v>
@@ -4369,7 +4386,7 @@
         <v>103</v>
       </c>
       <c r="L19" s="16" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="M19" s="16" t="s">
         <v>157</v>
@@ -4414,7 +4431,7 @@
         <v>97</v>
       </c>
       <c r="I20" s="16" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J20" s="16"/>
       <c r="K20" s="16" t="s">
@@ -4427,17 +4444,17 @@
         <v>157</v>
       </c>
       <c r="N20" s="16" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="O20" s="16" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="P20" s="16" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="Q20" s="16"/>
       <c r="R20" s="16" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="S20" s="16"/>
       <c r="T20" s="15" t="s">
@@ -4468,7 +4485,7 @@
         <v>107</v>
       </c>
       <c r="I21" s="16" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="J21" s="15" t="s">
         <v>99</v>
@@ -4479,7 +4496,7 @@
         <v>157</v>
       </c>
       <c r="N21" s="16" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="O21" s="16" t="s">
         <v>116</v>

</xml_diff>